<commit_message>
API request added products
</commit_message>
<xml_diff>
--- a/wp-content/themes/eurofert-theme/scripts/products.xlsx
+++ b/wp-content/themes/eurofert-theme/scripts/products.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\eurofert\wp-content\themes\eurofert-theme\scripts\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{852A314A-6975-49CC-9D36-200DC68EBD81}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E8ACE77-1E9F-49CA-B4B9-BFDDDCBF0837}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{76D0BCB8-E73B-4392-8B84-A7325E8578D8}"/>
   </bookViews>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="30">
   <si>
     <t>title</t>
   </si>
@@ -92,9 +92,6 @@
     <t xml:space="preserve">0-0-36+ 50% </t>
   </si>
   <si>
-    <t>K2O | 36.0 \n Organic Matter 50.0</t>
-  </si>
-  <si>
     <t>Enhances fruit size, sugar content, and color development\n Improves soil properties, buffering capacity, and microbial activity.\nIncreases plant vitality, vigor, and disease resistance.</t>
   </si>
   <si>
@@ -111,6 +108,23 @@
   </si>
   <si>
     <t>helps to balance the pH of alkaline spray solutions.</t>
+  </si>
+  <si>
+    <t>Colfert Essential PK</t>
+  </si>
+  <si>
+    <t>A fully water-soluble liquid fertilizer providing high concentrations of Phosphorus and Potassium.
+It enhances flower initiation, fruit size, and total solids, while improving plant resilience to stress, disease, and unfavorable growing conditions.</t>
+  </si>
+  <si>
+    <t>0-33-44</t>
+  </si>
+  <si>
+    <t>P2O5 | 33%
+K2O  | 44%</t>
+  </si>
+  <si>
+    <t>K2O | 36.0 \n Organic Matter |50.0</t>
   </si>
 </sst>
 </file>
@@ -980,7 +994,7 @@
     <col min="1" max="1" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15.88671875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="30.44140625" customWidth="1"/>
-    <col min="4" max="4" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="25.109375" style="1" customWidth="1"/>
     <col min="6" max="6" width="41.5546875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="32.77734375" customWidth="1"/>
@@ -1072,13 +1086,13 @@
         <v>colfert-essential-ktc.webp</v>
       </c>
       <c r="G3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H3" t="s">
         <v>18</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="J3" s="1" t="str">
         <f>IF(B3="","", B3 &amp; ".json")</f>
@@ -1087,87 +1101,116 @@
     </row>
     <row r="4" spans="1:10" ht="24" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B4" t="str">
-        <f t="shared" ref="B4:B20" si="0">SUBSTITUTE(LOWER(A4), " ", "-")</f>
+        <f t="shared" ref="B4:B5" si="0">SUBSTITUTE(LOWER(A4), " ", "-")</f>
         <v>colfert-essential-p</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D4" t="s">
         <v>15</v>
       </c>
       <c r="E4" s="1" t="str">
-        <f>IF(B4="","", B4 &amp; ".webp")</f>
+        <f t="shared" ref="E4:E5" si="1">IF(B4="","", B4 &amp; ".webp")</f>
         <v>colfert-essential-p.webp</v>
       </c>
       <c r="F4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="I4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="J4" s="1" t="str">
         <f>IF(B4="","", B4 &amp; ".json")</f>
         <v>colfert-essential-p.json</v>
       </c>
     </row>
+    <row r="5" spans="1:10" ht="115.2" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>colfert-essential-pk</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>colfert-essential-pk.webp</v>
+      </c>
+      <c r="H5" t="s">
+        <v>27</v>
+      </c>
+      <c r="I5" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J5" s="1" t="str">
+        <f>IF(B5="","", B5 &amp; ".json")</f>
+        <v>colfert-essential-pk.json</v>
+      </c>
+    </row>
     <row r="22" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D22" t="str">
-        <f t="shared" ref="D4:D30" si="1">SUBSTITUTE(LOWER(A22), " ", "-")</f>
+        <f t="shared" ref="D22:D30" si="2">SUBSTITUTE(LOWER(A22), " ", "-")</f>
         <v/>
       </c>
     </row>
     <row r="23" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D23" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="24" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D24" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="25" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D25" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="26" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D26" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="27" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D27" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="28" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D28" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="29" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D29" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>
     <row r="30" spans="4:4" x14ac:dyDescent="0.3">
       <c r="D30" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v/>
       </c>
     </row>

</xml_diff>